<commit_message>
LUXBIOTECH e LUXBIOTECH_EMS_HPC no lugar da EMS_OTC, e cota por hora a 95
As duas linhas novas da ENVIO MAPA.xlsx, semanal de segunda e mensal: LUXBIOTECH (61596,
Yuri, roberto.mattos@ems.com.br) e LUXBIOTECH_EMS_HPC (44421, 58532 e 47228 num relatorio
so, Joici, claudio.mendonca@legrandpharma.com.br). A EMS_OTC sai: os codigos dela passam
para a LUXBIOTECH_EMS_HPC. O 5853 da planilha nao existe no Geweb e foi lido como 58532.

Sao 48 laboratorios ativos; o pior caso (mensal atrasado recuperado numa segunda) vai a
48 + 47 = 95, e a cota por hora sobe de 93 para 95. Com os 2 e-mails da revisao sao 97
dos 100 por hora da Locaweb.
</commit_message>
<xml_diff>
--- a/docs/referencia/ENVIO MAPA.xlsx
+++ b/docs/referencia/ENVIO MAPA.xlsx
@@ -1,26 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro.veloso\Documents\Desenvolvimento - Interno\mapa-de-estoque\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro.veloso\Documents\Desenvolvimento - Interno\mapa-de-estoque\docs\referencia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5422DE41-C7E6-4617-A5F4-389B67593F90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29805963-5FF3-4E14-98C4-72DF57D4FF47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Worksheet!$A$1:$J$1</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="111">
   <si>
     <t>ID FABRICANTE</t>
   </si>
@@ -341,13 +344,25 @@
   </si>
   <si>
     <t>marilene.eduardo@catarinensepharma.com.br</t>
+  </si>
+  <si>
+    <t>claudio.mendonca@legrandpharma.com.br</t>
+  </si>
+  <si>
+    <t>LUXBIOTECH (EMS HPC)</t>
+  </si>
+  <si>
+    <t>LUXBIOTECH</t>
+  </si>
+  <si>
+    <t>44421 - 5853 -47228</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -365,12 +380,6 @@
       <color rgb="FF000000"/>
       <name val="Aptos Display"/>
       <family val="2"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <sz val="10"/>
@@ -405,7 +414,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -415,6 +424,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -443,11 +458,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -464,57 +478,56 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF92D050"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -814,17 +827,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="50.5546875" style="19" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="71.109375" style="14" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.6640625" style="1" customWidth="1"/>
     <col min="5" max="5" width="11.88671875" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.88671875" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.88671875" style="1" customWidth="1"/>
     <col min="10" max="10" width="40.109375" style="1" bestFit="1" customWidth="1"/>
   </cols>
@@ -833,7 +846,7 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
@@ -862,203 +875,203 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="16">
+        <v>46961</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" s="16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="16">
+        <v>61724</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="J3" s="16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="16">
+        <v>46239</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
+      <c r="I4" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" s="16" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="16">
+        <v>5660</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="J5" s="16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="16">
+        <v>61596</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>109</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="J6" s="16" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="16">
+        <v>39010</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="J7" s="16" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="16">
+        <v>44425</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="J8" s="16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="J9" s="16" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B10" s="4" t="s">
         <v>11</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="3">
-        <v>106499</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="3">
-        <v>7142</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="3">
-        <v>122992</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="3">
-        <v>123174</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="3">
-        <v>22999</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="3">
-        <v>46961</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="3">
-        <v>61724</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>22</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>12</v>
@@ -1074,15 +1087,15 @@
         <v>13</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="3">
-        <v>46239</v>
+      <c r="A11" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>12</v>
@@ -1097,16 +1110,16 @@
       <c r="I11" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J11" s="3" t="s">
-        <v>25</v>
+      <c r="J11" s="5" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
-        <v>14232</v>
+        <v>106499</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>12</v>
@@ -1121,16 +1134,16 @@
       <c r="I12" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J12" s="3" t="s">
-        <v>27</v>
+      <c r="J12" s="5" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
-        <v>13963</v>
+        <v>7142</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>12</v>
@@ -1139,24 +1152,22 @@
         <v>13</v>
       </c>
       <c r="E13" s="3"/>
-      <c r="F13" s="3" t="s">
-        <v>13</v>
-      </c>
+      <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J13" s="3" t="s">
-        <v>28</v>
+      <c r="J13" s="5" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
-        <v>5660</v>
+        <v>122992</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>12</v>
@@ -1172,15 +1183,15 @@
         <v>13</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>23</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
-        <v>40333</v>
+        <v>123174</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>12</v>
@@ -1195,16 +1206,16 @@
       <c r="I15" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J15" s="6" t="s">
-        <v>79</v>
+      <c r="J15" s="3" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
-        <v>30314</v>
+        <v>22999</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>12</v>
@@ -1220,15 +1231,15 @@
         <v>13</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
-        <v>39010</v>
+        <v>14232</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>12</v>
@@ -1244,15 +1255,15 @@
         <v>13</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
-        <v>44425</v>
+        <v>13963</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>12</v>
@@ -1261,22 +1272,24 @@
         <v>13</v>
       </c>
       <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
+      <c r="F18" s="3" t="s">
+        <v>13</v>
+      </c>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
       <c r="I18" s="3" t="s">
         <v>13</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
-        <v>7127</v>
+        <v>40333</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>12</v>
@@ -1285,24 +1298,22 @@
         <v>13</v>
       </c>
       <c r="E19" s="3"/>
-      <c r="F19" s="3" t="s">
-        <v>13</v>
-      </c>
+      <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
       <c r="I19" s="3" t="s">
         <v>13</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>36</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
-        <v>47658</v>
+        <v>30314</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>12</v>
@@ -1318,15 +1329,15 @@
         <v>13</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
-        <v>104634</v>
+        <v>7127</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>12</v>
@@ -1335,22 +1346,24 @@
         <v>13</v>
       </c>
       <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
+      <c r="F21" s="3" t="s">
+        <v>13</v>
+      </c>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
       <c r="I21" s="3" t="s">
         <v>13</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="3">
-        <v>52878</v>
+        <v>47658</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>12</v>
@@ -1366,15 +1379,15 @@
         <v>13</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
-        <v>58650</v>
+        <v>104634</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>12</v>
@@ -1390,15 +1403,15 @@
         <v>13</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24" s="3" t="s">
-        <v>45</v>
+      <c r="A24" s="3">
+        <v>52878</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>12</v>
@@ -1414,15 +1427,15 @@
         <v>13</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="3">
-        <v>46292</v>
+        <v>58650</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>12</v>
@@ -1438,18 +1451,18 @@
         <v>13</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A26" s="3">
-        <v>7485</v>
+      <c r="A26" s="3" t="s">
+        <v>45</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>56</v>
+        <v>12</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>13</v>
@@ -1461,19 +1474,19 @@
       <c r="I26" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J26" s="6" t="s">
-        <v>57</v>
+      <c r="J26" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
-        <v>23975</v>
+        <v>46292</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>56</v>
+        <v>12</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>13</v>
@@ -1485,16 +1498,16 @@
       <c r="I27" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J27" s="7" t="s">
-        <v>59</v>
+      <c r="J27" s="3" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="3">
-        <v>43176</v>
+        <v>7485</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>56</v>
@@ -1509,252 +1522,252 @@
       <c r="I28" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J28" s="7" t="s">
+      <c r="J28" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A29" s="3">
+        <v>23975</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A30" s="3">
+        <v>43176</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J30" s="3" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A29" s="8">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A31" s="6">
         <v>47476</v>
       </c>
-      <c r="B29" s="9" t="s">
+      <c r="B31" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C31" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="D29" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="E29" s="8"/>
-      <c r="F29" s="8"/>
-      <c r="G29" s="8"/>
-      <c r="H29" s="8"/>
-      <c r="I29" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J29" s="6" t="s">
+      <c r="D31" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J31" s="3" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A30" s="8">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A32" s="6">
         <v>107151</v>
       </c>
-      <c r="B30" s="12" t="s">
+      <c r="B32" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="C32" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="D30" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="E30" s="8"/>
-      <c r="F30" s="8"/>
-      <c r="G30" s="8"/>
-      <c r="H30" s="8"/>
-      <c r="I30" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J30" s="11" t="s">
+      <c r="D32" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E32" s="6"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="6"/>
+      <c r="H32" s="6"/>
+      <c r="I32" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J32" s="3" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A31" s="8">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A33" s="6">
         <v>49913</v>
       </c>
-      <c r="B31" s="9" t="s">
+      <c r="B33" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C33" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="D31" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="E31" s="8"/>
-      <c r="F31" s="8"/>
-      <c r="G31" s="8"/>
-      <c r="H31" s="8"/>
-      <c r="I31" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J31" s="11" t="s">
+      <c r="D33" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="6"/>
+      <c r="H33" s="6"/>
+      <c r="I33" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J33" s="3" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A32" s="8">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A34" s="6">
         <v>45484</v>
       </c>
-      <c r="B32" s="9" t="s">
+      <c r="B34" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C32" s="10" t="s">
+      <c r="C34" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="D32" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="E32" s="8"/>
-      <c r="F32" s="8"/>
-      <c r="G32" s="8"/>
-      <c r="H32" s="8"/>
-      <c r="I32" s="8"/>
-      <c r="J32" s="11" t="s">
+      <c r="D34" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E34" s="6"/>
+      <c r="F34" s="6"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="6"/>
+      <c r="I34" s="6"/>
+      <c r="J34" s="3" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A33" s="8">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A35" s="6">
         <v>22866</v>
       </c>
-      <c r="B33" s="9" t="s">
+      <c r="B35" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="C33" s="10" t="s">
+      <c r="C35" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="D33" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="E33" s="8"/>
-      <c r="F33" s="8"/>
-      <c r="G33" s="8"/>
-      <c r="H33" s="8"/>
-      <c r="I33" s="8"/>
-      <c r="J33" s="11" t="s">
+      <c r="D35" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E35" s="6"/>
+      <c r="F35" s="6"/>
+      <c r="G35" s="6"/>
+      <c r="H35" s="6"/>
+      <c r="I35" s="6"/>
+      <c r="J35" s="3" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A34" s="8">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A36" s="6">
         <v>21729</v>
       </c>
-      <c r="B34" s="9" t="s">
+      <c r="B36" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C34" s="10" t="s">
+      <c r="C36" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="D34" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="E34" s="8"/>
-      <c r="F34" s="8"/>
-      <c r="G34" s="8"/>
-      <c r="H34" s="8"/>
-      <c r="I34" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J34" s="11" t="s">
+      <c r="D36" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="6"/>
+      <c r="H36" s="6"/>
+      <c r="I36" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J36" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A35" s="10" t="s">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A37" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B35" s="9" t="s">
+      <c r="B37" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C35" s="10" t="s">
+      <c r="C37" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="D35" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="E35" s="8"/>
-      <c r="F35" s="8"/>
-      <c r="G35" s="8"/>
-      <c r="H35" s="8"/>
-      <c r="I35" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J35" s="11" t="s">
+      <c r="D37" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+      <c r="I37" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J37" s="9" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A36" s="8">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A38" s="6">
         <v>27878</v>
       </c>
-      <c r="B36" s="9" t="s">
+      <c r="B38" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="C36" s="10" t="s">
+      <c r="C38" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="D36" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="E36" s="8"/>
-      <c r="F36" s="8"/>
-      <c r="G36" s="8"/>
-      <c r="H36" s="8"/>
-      <c r="I36" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J36" s="11" t="s">
+      <c r="D38" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E38" s="6"/>
+      <c r="F38" s="6"/>
+      <c r="G38" s="6"/>
+      <c r="H38" s="6"/>
+      <c r="I38" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J38" s="9" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A37" s="3">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A39" s="3">
         <v>35729</v>
       </c>
-      <c r="B37" s="17" t="s">
+      <c r="B39" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="D37" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E37" s="3"/>
-      <c r="F37" s="3"/>
-      <c r="G37" s="3"/>
-      <c r="H37" s="3"/>
-      <c r="I37" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J37" s="13" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A38" s="3">
-        <v>7181</v>
-      </c>
-      <c r="B38" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="D38" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E38" s="3"/>
-      <c r="F38" s="3"/>
-      <c r="G38" s="3"/>
-      <c r="H38" s="3"/>
-      <c r="I38" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J38" s="13" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A39" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="B39" s="17" t="s">
-        <v>86</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>82</v>
@@ -1769,16 +1782,16 @@
       <c r="I39" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J39" s="13" t="s">
-        <v>87</v>
+      <c r="J39" s="9" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="3">
-        <v>19117</v>
-      </c>
-      <c r="B40" s="17" t="s">
-        <v>88</v>
+        <v>7181</v>
+      </c>
+      <c r="B40" s="12" t="s">
+        <v>84</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>82</v>
@@ -1793,16 +1806,16 @@
       <c r="I40" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J40" s="14" t="s">
-        <v>89</v>
+      <c r="J40" s="9" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B41" s="17" t="s">
-        <v>91</v>
+        <v>85</v>
+      </c>
+      <c r="B41" s="12" t="s">
+        <v>86</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>82</v>
@@ -1817,16 +1830,16 @@
       <c r="I41" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J41" s="15" t="s">
-        <v>92</v>
+      <c r="J41" s="9" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="3">
-        <v>20285</v>
-      </c>
-      <c r="B42" s="17" t="s">
-        <v>93</v>
+        <v>19117</v>
+      </c>
+      <c r="B42" s="12" t="s">
+        <v>88</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>82</v>
@@ -1841,16 +1854,16 @@
       <c r="I42" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J42" s="7" t="s">
-        <v>106</v>
+      <c r="J42" s="9" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A43" s="3">
-        <v>22287</v>
-      </c>
-      <c r="B43" s="17" t="s">
-        <v>94</v>
+      <c r="A43" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B43" s="12" t="s">
+        <v>91</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>82</v>
@@ -1865,16 +1878,16 @@
       <c r="I43" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J43" s="13" t="s">
-        <v>95</v>
+      <c r="J43" s="9" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="3">
-        <v>27499</v>
-      </c>
-      <c r="B44" s="17" t="s">
-        <v>96</v>
+        <v>20285</v>
+      </c>
+      <c r="B44" s="12" t="s">
+        <v>93</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>82</v>
@@ -1889,16 +1902,16 @@
       <c r="I44" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J44" s="13" t="s">
-        <v>78</v>
+      <c r="J44" s="9" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A45" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B45" s="17" t="s">
-        <v>98</v>
+      <c r="A45" s="3">
+        <v>22287</v>
+      </c>
+      <c r="B45" s="12" t="s">
+        <v>94</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>82</v>
@@ -1913,16 +1926,16 @@
       <c r="I45" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J45" s="7" t="s">
-        <v>99</v>
+      <c r="J45" s="9" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A46" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="B46" s="17" t="s">
-        <v>101</v>
+      <c r="A46" s="3">
+        <v>27499</v>
+      </c>
+      <c r="B46" s="12" t="s">
+        <v>96</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>82</v>
@@ -1934,17 +1947,19 @@
       <c r="F46" s="3"/>
       <c r="G46" s="3"/>
       <c r="H46" s="3"/>
-      <c r="I46" s="3"/>
-      <c r="J46" s="13" t="s">
-        <v>102</v>
+      <c r="I46" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J46" s="9" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="B47" s="18" t="s">
-        <v>103</v>
+        <v>97</v>
+      </c>
+      <c r="B47" s="12" t="s">
+        <v>98</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>82</v>
@@ -1959,30 +1974,83 @@
       <c r="I47" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J47" s="7" t="s">
+      <c r="J47" s="9" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A48" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B48" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+      <c r="I48" s="3"/>
+      <c r="J48" s="9" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A49" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B49" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E49" s="3"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
+      <c r="I49" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J49" s="9" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="50" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D50" s="20"/>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D52" s="15"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:J1" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J51">
+      <sortCondition sortBy="cellColor" ref="B1" dxfId="0"/>
+    </sortState>
+  </autoFilter>
   <hyperlinks>
-    <hyperlink ref="J6" r:id="rId1" xr:uid="{9791F816-AA06-4D59-AED6-32837D568F3D}"/>
-    <hyperlink ref="J7" r:id="rId2" xr:uid="{232E5092-F983-4133-A14B-FEF596F279D2}"/>
-    <hyperlink ref="J25" r:id="rId3" xr:uid="{5249B9AE-EB38-4E91-BFD1-3D2B5D840CC0}"/>
-    <hyperlink ref="J26" r:id="rId4" xr:uid="{102A299D-9405-467D-A338-99BE13828AE8}"/>
-    <hyperlink ref="J27" r:id="rId5" xr:uid="{0CA6C4B7-6F96-42FC-8784-88994DB3A77D}"/>
-    <hyperlink ref="J28" r:id="rId6" xr:uid="{9AA2C8E6-8A1C-4371-859B-ACD40B39CFC6}"/>
-    <hyperlink ref="J30" r:id="rId7" xr:uid="{5ACA3C95-40B7-46A6-8537-5D1484E9D1C0}"/>
-    <hyperlink ref="J15" r:id="rId8" xr:uid="{6F0B471E-DB43-4334-AC70-44E5463FD9DD}"/>
-    <hyperlink ref="J29" r:id="rId9" xr:uid="{89386F5F-DC0B-4223-B9AA-DCB36A628539}"/>
-    <hyperlink ref="J37" r:id="rId10" xr:uid="{D61F6EC0-90F6-440D-89EA-18716E977648}"/>
-    <hyperlink ref="J38" r:id="rId11" xr:uid="{A2B9810A-E68E-45AD-9268-07BC0A06E8F7}"/>
-    <hyperlink ref="J42" r:id="rId12" xr:uid="{F8B32B5D-3A34-4EFD-B3A0-B496AD2F74EB}"/>
-    <hyperlink ref="J43" r:id="rId13" xr:uid="{F14AD8A1-C901-43CB-8A87-667222469056}"/>
-    <hyperlink ref="J45" r:id="rId14" xr:uid="{5985511B-5A12-447A-B36C-8FA973F88D90}"/>
-    <hyperlink ref="J47" r:id="rId15" xr:uid="{285DDA20-E050-4D54-91A6-6F4C937F2634}"/>
+    <hyperlink ref="J14" r:id="rId1" xr:uid="{9791F816-AA06-4D59-AED6-32837D568F3D}"/>
+    <hyperlink ref="J15" r:id="rId2" xr:uid="{232E5092-F983-4133-A14B-FEF596F279D2}"/>
+    <hyperlink ref="J27" r:id="rId3" xr:uid="{5249B9AE-EB38-4E91-BFD1-3D2B5D840CC0}"/>
+    <hyperlink ref="J28" r:id="rId4" xr:uid="{102A299D-9405-467D-A338-99BE13828AE8}"/>
+    <hyperlink ref="J29" r:id="rId5" xr:uid="{0CA6C4B7-6F96-42FC-8784-88994DB3A77D}"/>
+    <hyperlink ref="J30" r:id="rId6" xr:uid="{9AA2C8E6-8A1C-4371-859B-ACD40B39CFC6}"/>
+    <hyperlink ref="J32" r:id="rId7" xr:uid="{5ACA3C95-40B7-46A6-8537-5D1484E9D1C0}"/>
+    <hyperlink ref="J19" r:id="rId8" xr:uid="{6F0B471E-DB43-4334-AC70-44E5463FD9DD}"/>
+    <hyperlink ref="J31" r:id="rId9" xr:uid="{89386F5F-DC0B-4223-B9AA-DCB36A628539}"/>
+    <hyperlink ref="J39" r:id="rId10" xr:uid="{D61F6EC0-90F6-440D-89EA-18716E977648}"/>
+    <hyperlink ref="J40" r:id="rId11" xr:uid="{A2B9810A-E68E-45AD-9268-07BC0A06E8F7}"/>
+    <hyperlink ref="J44" r:id="rId12" xr:uid="{F8B32B5D-3A34-4EFD-B3A0-B496AD2F74EB}"/>
+    <hyperlink ref="J45" r:id="rId13" xr:uid="{F14AD8A1-C901-43CB-8A87-667222469056}"/>
+    <hyperlink ref="J47" r:id="rId14" xr:uid="{5985511B-5A12-447A-B36C-8FA973F88D90}"/>
+    <hyperlink ref="J49" r:id="rId15" xr:uid="{285DDA20-E050-4D54-91A6-6F4C937F2634}"/>
+    <hyperlink ref="J9" r:id="rId16" xr:uid="{F0836C89-8988-4737-A69D-6095E033A462}"/>
+    <hyperlink ref="J6" r:id="rId17" xr:uid="{ADF9A038-E997-401A-84D7-64A703E66424}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>